<commit_message>
Update test samples and input
</commit_message>
<xml_diff>
--- a/day0.xlsx
+++ b/day0.xlsx
@@ -413,9 +413,690 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:V10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1" t="n">
+        <v>201917</v>
+      </c>
+      <c r="G1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1" t="n">
+        <v>999</v>
+      </c>
+      <c r="J1" t="n">
+        <v>999</v>
+      </c>
+      <c r="K1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O1" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="P1" t="n">
+        <v>29.48256</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R1" t="n">
+        <v>2</v>
+      </c>
+      <c r="S1" t="n">
+        <v>1500</v>
+      </c>
+      <c r="T1" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U1" t="n">
+        <v>100</v>
+      </c>
+      <c r="V1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>201917</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>999</v>
+      </c>
+      <c r="J2" t="n">
+        <v>999</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="P2" t="n">
+        <v>29.48256</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U2" t="n">
+        <v>100</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>201917</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>999</v>
+      </c>
+      <c r="J3" t="n">
+        <v>999</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="P3" t="n">
+        <v>29.48256</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S3" t="n">
+        <v>1500</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U3" t="n">
+        <v>100</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>201917</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>999</v>
+      </c>
+      <c r="J4" t="n">
+        <v>999</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="P4" t="n">
+        <v>29.48256</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U4" t="n">
+        <v>100</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>201917</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>999</v>
+      </c>
+      <c r="J5" t="n">
+        <v>999</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="P5" t="n">
+        <v>29.48256</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U5" t="n">
+        <v>100</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>201917</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>999</v>
+      </c>
+      <c r="J6" t="n">
+        <v>999</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="P6" t="n">
+        <v>29.48256</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>2</v>
+      </c>
+      <c r="S6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U6" t="n">
+        <v>100</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>201917</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>999</v>
+      </c>
+      <c r="J7" t="n">
+        <v>999</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="P7" t="n">
+        <v>29.48256</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>2</v>
+      </c>
+      <c r="S7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U7" t="n">
+        <v>100</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>201917</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>999</v>
+      </c>
+      <c r="J8" t="n">
+        <v>999</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="P8" t="n">
+        <v>29.48256</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U8" t="n">
+        <v>100</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>201917</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>999</v>
+      </c>
+      <c r="J9" t="n">
+        <v>999</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="P9" t="n">
+        <v>29.48256</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>2</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U9" t="n">
+        <v>100</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>201917</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>999</v>
+      </c>
+      <c r="J10" t="n">
+        <v>999</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="P10" t="n">
+        <v>29.48256</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U10" t="n">
+        <v>100</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>